<commit_message>
Adjust the fiberport class and update the production folder
</commit_message>
<xml_diff>
--- a/Production/LaserBoard/Laser_Board.xlsx
+++ b/Production/LaserBoard/Laser_Board.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Augenblick/Documents/2025Summer/FreeCAD/Boards/PyOpticL_Rubidium_System/Production/LaserBoard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AA77CC-58AA-DD49-A03A-7F8BD6805C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5C9E5E-1A9E-3145-8923-28D091DCCB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1260" yWindow="680" windowWidth="28040" windowHeight="17440" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
@@ -517,7 +517,7 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Redesigned the board combinations and usage to reduce the number of board types.
</commit_message>
<xml_diff>
--- a/Production/LaserBoard/Laser_Board.xlsx
+++ b/Production/LaserBoard/Laser_Board.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Augenblick/Documents/2025Summer/FreeCAD/Boards/PyOpticL_Rubidium_System/Production/LaserBoard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5C9E5E-1A9E-3145-8923-28D091DCCB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE64EC8-F55F-BC44-AEE2-C0CF62508A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1260" yWindow="680" windowWidth="28040" windowHeight="17440" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Adaptors</t>
   </si>
@@ -55,6 +55,9 @@
     <t>Surface_Adapter_fiberport_lip.step</t>
   </si>
   <si>
+    <t>Cube_Mount.step</t>
+  </si>
+  <si>
     <t>KM05T</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>cube</t>
   </si>
   <si>
-    <t>Laser_baseboard.step</t>
+    <t>MOT_baseboard.step</t>
   </si>
   <si>
     <t>Laser Board</t>
@@ -477,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504A0317-4413-EE44-9F8B-28AC1E65744B}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -485,7 +488,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -506,7 +509,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -517,7 +520,7 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -525,7 +528,7 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -533,31 +536,31 @@
         <v>5</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13">
-        <v>4</v>
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -565,28 +568,28 @@
         <v>11</v>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -597,7 +600,7 @@
         <v>8</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -605,15 +608,15 @@
         <v>9</v>
       </c>
       <c r="B19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -621,28 +624,36 @@
         <v>13</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>17</v>
+      <c r="A22" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A18" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
-    <hyperlink ref="A19" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
-    <hyperlink ref="A15" r:id="rId3" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=KM05T" xr:uid="{1BBCBD75-E5E4-9C42-9870-10D5AFE8751D}"/>
-    <hyperlink ref="A13" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
-    <hyperlink ref="A14" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=IO-3D-780-VLP" xr:uid="{27DD0994-D2B1-854C-8165-72C16DCFC984}"/>
-    <hyperlink ref="A20" r:id="rId6" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
-    <hyperlink ref="A21" r:id="rId7" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
-    <hyperlink ref="A16" r:id="rId8" xr:uid="{103D64FF-9059-1B42-816A-F92B0274781E}"/>
-    <hyperlink ref="A17" r:id="rId9" xr:uid="{CA5CFB4E-909E-4340-8D31-B44B7990E725}"/>
+    <hyperlink ref="A19" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
+    <hyperlink ref="A20" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
+    <hyperlink ref="A16" r:id="rId3" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=KM05T" xr:uid="{1BBCBD75-E5E4-9C42-9870-10D5AFE8751D}"/>
+    <hyperlink ref="A14" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
+    <hyperlink ref="A15" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=IO-3D-780-VLP" xr:uid="{27DD0994-D2B1-854C-8165-72C16DCFC984}"/>
+    <hyperlink ref="A21" r:id="rId6" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
+    <hyperlink ref="A22" r:id="rId7" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
+    <hyperlink ref="A17" r:id="rId8" xr:uid="{103D64FF-9059-1B42-816A-F92B0274781E}"/>
+    <hyperlink ref="A18" r:id="rId9" xr:uid="{CA5CFB4E-909E-4340-8D31-B44B7990E725}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Revised parts spreadsheet, replaced KA05TB by KA05T
</commit_message>
<xml_diff>
--- a/Production/LaserBoard/Laser_Board.xlsx
+++ b/Production/LaserBoard/Laser_Board.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Augenblick/Documents/2025Summer/FreeCAD/Boards/PyOpticL_Rubidium_System/Production/LaserBoard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Github/PyOpticL_Rubidium_System/Production/LaserBoard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE64EC8-F55F-BC44-AEE2-C0CF62508A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD1FE70-28FB-ED4E-8F28-3526D8EA8174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
+    <workbookView xWindow="19400" yWindow="740" windowWidth="10000" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>Cube_Mount.step</t>
   </si>
   <si>
-    <t>KM05T</t>
-  </si>
-  <si>
     <t>M05</t>
   </si>
   <si>
@@ -98,6 +95,9 @@
   </si>
   <si>
     <t>Laser Board</t>
+  </si>
+  <si>
+    <t>KA05T</t>
   </si>
 </sst>
 </file>
@@ -488,7 +488,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -509,7 +509,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -549,7 +549,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
         <v>1</v>
@@ -565,7 +565,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14">
         <v>7</v>
@@ -573,7 +573,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -581,7 +581,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B16">
         <v>2</v>
@@ -589,7 +589,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17">
         <v>1</v>
@@ -597,15 +597,15 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B18">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -613,7 +613,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>2</v>
@@ -621,7 +621,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21">
         <v>2</v>
@@ -629,7 +629,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B22">
         <v>2</v>
@@ -637,17 +637,17 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A19" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
     <hyperlink ref="A20" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
-    <hyperlink ref="A16" r:id="rId3" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=KM05T" xr:uid="{1BBCBD75-E5E4-9C42-9870-10D5AFE8751D}"/>
+    <hyperlink ref="A16" r:id="rId3" xr:uid="{1BBCBD75-E5E4-9C42-9870-10D5AFE8751D}"/>
     <hyperlink ref="A14" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
     <hyperlink ref="A15" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=IO-3D-780-VLP" xr:uid="{27DD0994-D2B1-854C-8165-72C16DCFC984}"/>
     <hyperlink ref="A21" r:id="rId6" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>

</xml_diff>

<commit_message>
Updated parts list, picture, Step files, Baseplate files
</commit_message>
<xml_diff>
--- a/Production/LaserBoard/Laser_Board.xlsx
+++ b/Production/LaserBoard/Laser_Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Github/PyOpticL_Rubidium_System/Production/LaserBoard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD1FE70-28FB-ED4E-8F28-3526D8EA8174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A693BC-8211-6D41-AD73-9059C174AE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19400" yWindow="740" windowWidth="10000" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
@@ -91,13 +91,13 @@
     <t>cube</t>
   </si>
   <si>
-    <t>MOT_baseboard.step</t>
-  </si>
-  <si>
     <t>Laser Board</t>
   </si>
   <si>
     <t>KA05T</t>
+  </si>
+  <si>
+    <t>Laser_Baseplate1.step</t>
   </si>
 </sst>
 </file>
@@ -488,7 +488,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -549,7 +549,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -581,7 +581,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16">
         <v>2</v>

</xml_diff>